<commit_message>
add keywords, replce spec sheets
</commit_message>
<xml_diff>
--- a/public/files/spec.xlsx
+++ b/public/files/spec.xlsx
@@ -8,19 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\박승범\Desktop\sekyungnet-nextjs\public\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5FB1DE1-A8C2-449E-BFBB-9BF504746017}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA5A7335-18EA-4B01-B22C-388E0002784E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8670" yWindow="0" windowWidth="18600" windowHeight="15585" xr2:uid="{3815D4BE-58CE-4EF9-83C9-4D98FA1B59A4}"/>
+    <workbookView xWindow="5250" yWindow="0" windowWidth="21825" windowHeight="15165" xr2:uid="{3815D4BE-58CE-4EF9-83C9-4D98FA1B59A4}"/>
   </bookViews>
   <sheets>
-    <sheet name="spec" sheetId="1" r:id="rId1"/>
+    <sheet name="specs" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0" iterate="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="55">
   <si>
     <t>PLY</t>
   </si>
@@ -79,18 +79,12 @@
     <t>ceiling net</t>
   </si>
   <si>
-    <t>4ply</t>
-  </si>
-  <si>
     <t>UHMWPE</t>
   </si>
   <si>
     <t>baseball</t>
   </si>
   <si>
-    <t>8ply</t>
-  </si>
-  <si>
     <t>210ply</t>
   </si>
   <si>
@@ -100,9 +94,6 @@
     <t>baseball/football net</t>
   </si>
   <si>
-    <t>MD</t>
-  </si>
-  <si>
     <t>Kg</t>
   </si>
   <si>
@@ -116,9 +107,6 @@
   </si>
   <si>
     <t>HTPE(High Tenacity PE)</t>
-  </si>
-  <si>
-    <t>Available Product Specifications</t>
   </si>
   <si>
     <t>Twisted Knotless Net (Sports Net, Square Mesh)</t>
@@ -229,6 +217,26 @@
     <t>baseball / tennis / football net</t>
     <phoneticPr fontId="19" type="noConversion"/>
   </si>
+  <si>
+    <t>10ply</t>
+    <phoneticPr fontId="19" type="noConversion"/>
+  </si>
+  <si>
+    <t>16ply</t>
+    <phoneticPr fontId="19" type="noConversion"/>
+  </si>
+  <si>
+    <t>golf net</t>
+    <phoneticPr fontId="19" type="noConversion"/>
+  </si>
+  <si>
+    <t>MD</t>
+    <phoneticPr fontId="19" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">        Available Product Specifications</t>
+    <phoneticPr fontId="19" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
@@ -424,8 +432,9 @@
       <charset val="129"/>
     </font>
     <font>
+      <b/>
       <sz val="14"/>
-      <color rgb="FF0070C0"/>
+      <color rgb="FF2DB958"/>
       <name val="Malgun Gothic"/>
       <family val="3"/>
       <charset val="129"/>
@@ -618,7 +627,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -794,21 +803,78 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
       <bottom style="medium">
         <color rgb="FFCCCCCC"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
       <top style="medium">
         <color rgb="FFCCCCCC"/>
       </top>
-      <bottom/>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -940,7 +1006,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -949,38 +1015,44 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="18" fillId="33" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="18" fillId="33" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="18" fillId="33" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="18" fillId="33" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="33" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="33" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1029,6 +1101,11 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FF2DB958"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1348,12 +1425,12 @@
   <sheetData>
     <row r="1" spans="1:6" ht="33" customHeight="1">
       <c r="A1" s="3"/>
-      <c r="B1" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
+      <c r="B1" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
       <c r="F1" s="3"/>
     </row>
     <row r="2" spans="1:6">
@@ -1364,38 +1441,38 @@
       <c r="E2" s="3"/>
       <c r="F2" s="3"/>
     </row>
-    <row r="3" spans="1:6" ht="17.25" thickBot="1">
-      <c r="A3" s="18" t="s">
-        <v>33</v>
-      </c>
-      <c r="B3" s="7"/>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
-      <c r="F3" s="7"/>
-    </row>
-    <row r="4" spans="1:6" s="11" customFormat="1" ht="17.25" thickBot="1">
-      <c r="A4" s="8" t="s">
+    <row r="3" spans="1:6">
+      <c r="A3" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+    </row>
+    <row r="4" spans="1:6" s="4" customFormat="1" ht="17.25" thickBot="1">
+      <c r="A4" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="D4" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="F4" s="10" t="s">
+      <c r="E4" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="F4" s="11" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="17.25" thickBot="1">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="12" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="1" t="s">
@@ -1410,12 +1487,12 @@
       <c r="E5" s="2">
         <v>1.9</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="F5" s="13" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="17.25" thickBot="1">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="12" t="s">
         <v>6</v>
       </c>
       <c r="B6" s="1" t="s">
@@ -1430,12 +1507,12 @@
       <c r="E6" s="2">
         <v>1.9</v>
       </c>
-      <c r="F6" s="1" t="s">
-        <v>43</v>
+      <c r="F6" s="13" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="17.25" thickBot="1">
-      <c r="A7" s="1" t="s">
+      <c r="A7" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B7" s="1" t="s">
@@ -1450,12 +1527,12 @@
       <c r="E7" s="2">
         <v>2.1</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="F7" s="13" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="17.25" thickBot="1">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="12" t="s">
         <v>13</v>
       </c>
       <c r="B8" s="1" t="s">
@@ -1470,12 +1547,12 @@
       <c r="E8" s="2">
         <v>2.5</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="F8" s="13" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="17.25" thickBot="1">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="12" t="s">
         <v>16</v>
       </c>
       <c r="B9" s="1" t="s">
@@ -1490,12 +1567,12 @@
       <c r="E9" s="2">
         <v>3</v>
       </c>
-      <c r="F9" s="1" t="s">
-        <v>53</v>
+      <c r="F9" s="13" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="17.25" thickBot="1">
-      <c r="A10" s="1" t="s">
+      <c r="A10" s="12" t="s">
         <v>16</v>
       </c>
       <c r="B10" s="1" t="s">
@@ -1510,48 +1587,48 @@
       <c r="E10" s="2">
         <v>3</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="F10" s="13" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="17.25" thickBot="1">
-      <c r="A11" s="1" t="s">
+      <c r="A11" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B11" s="1" t="s">
-        <v>20</v>
-      </c>
       <c r="C11" s="1" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>9</v>
       </c>
       <c r="E11" s="2">
+        <v>0.8</v>
+      </c>
+      <c r="F11" s="13" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="B12" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="D12" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="E12" s="16">
         <v>1.2</v>
       </c>
-      <c r="F11" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="17.25" thickBot="1">
-      <c r="A12" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E12" s="2">
-        <v>1.9</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>21</v>
+      <c r="F12" s="17" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -1562,38 +1639,38 @@
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
     </row>
-    <row r="14" spans="1:6" ht="17.25" thickBot="1">
-      <c r="A14" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="B14" s="7"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
+    <row r="14" spans="1:6">
+      <c r="A14" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
     </row>
     <row r="15" spans="1:6" ht="17.25" thickBot="1">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="C15" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="D15" s="5" t="s">
+      <c r="D15" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="E15" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="F15" s="6" t="s">
+      <c r="E15" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="F15" s="20" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="17.25" thickBot="1">
-      <c r="A16" s="1" t="s">
+      <c r="A16" s="12" t="s">
         <v>13</v>
       </c>
       <c r="B16" s="1" t="s">
@@ -1608,13 +1685,13 @@
       <c r="E16" s="2">
         <v>2.5</v>
       </c>
-      <c r="F16" s="1" t="s">
+      <c r="F16" s="13" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="17.25" thickBot="1">
+      <c r="A17" s="12" t="s">
         <v>21</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" ht="17.25" thickBot="1">
-      <c r="A17" s="1" t="s">
-        <v>23</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>7</v>
@@ -1628,48 +1705,48 @@
       <c r="E17" s="2">
         <v>4.5</v>
       </c>
-      <c r="F17" s="1" t="s">
-        <v>24</v>
+      <c r="F17" s="13" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="17.25" thickBot="1">
-      <c r="A18" s="1" t="s">
+      <c r="A18" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="B18" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B18" s="1" t="s">
-        <v>20</v>
-      </c>
       <c r="C18" s="1" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>9</v>
       </c>
       <c r="E18" s="2">
+        <v>0.8</v>
+      </c>
+      <c r="F18" s="13" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
+      <c r="A19" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="B19" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="C19" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="D19" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="E19" s="16">
         <v>1.2</v>
       </c>
-      <c r="F18" s="1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" ht="17.25" thickBot="1">
-      <c r="A19" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E19" s="2">
-        <v>1.9</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>25</v>
+      <c r="F19" s="17" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -1680,113 +1757,113 @@
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
     </row>
-    <row r="21" spans="1:6" ht="17.25" thickBot="1">
-      <c r="A21" s="18" t="s">
-        <v>37</v>
-      </c>
-      <c r="B21" s="7"/>
-      <c r="C21" s="7"/>
-      <c r="D21" s="7"/>
-      <c r="E21" s="7"/>
-      <c r="F21" s="7"/>
+    <row r="21" spans="1:6">
+      <c r="A21" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B21" s="3"/>
+      <c r="C21" s="3"/>
+      <c r="D21" s="3"/>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
     </row>
     <row r="22" spans="1:6" ht="17.25" thickBot="1">
-      <c r="A22" s="4" t="s">
+      <c r="A22" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B22" s="5" t="s">
+      <c r="B22" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="C22" s="5" t="s">
+      <c r="C22" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="D22" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="E22" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F22" s="6" t="s">
+      <c r="D22" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="E22" s="19" t="s">
+        <v>24</v>
+      </c>
+      <c r="F22" s="20" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="17.25" thickBot="1">
-      <c r="A23" s="1" t="s">
+      <c r="A23" s="12" t="s">
         <v>6</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="E23" s="2">
         <v>150</v>
       </c>
-      <c r="F23" s="2">
+      <c r="F23" s="21">
         <v>1.9</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="17.25" thickBot="1">
-      <c r="A24" s="1" t="s">
+      <c r="A24" s="12" t="s">
         <v>13</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="E24" s="2">
         <v>225</v>
       </c>
-      <c r="F24" s="2">
+      <c r="F24" s="21">
         <v>2.5</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="17.25" thickBot="1">
-      <c r="A25" s="1" t="s">
+      <c r="A25" s="12" t="s">
         <v>16</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="E25" s="2">
         <v>150</v>
       </c>
-      <c r="F25" s="2">
+      <c r="F25" s="21">
         <v>3</v>
       </c>
     </row>
-    <row r="26" spans="1:6" ht="17.25" thickBot="1">
-      <c r="A26" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E26" s="2">
+    <row r="26" spans="1:6">
+      <c r="A26" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="B26" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C26" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="D26" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="E26" s="16">
         <v>150</v>
       </c>
-      <c r="F26" s="1">
+      <c r="F26" s="17">
         <v>1.9</v>
       </c>
     </row>
@@ -1798,95 +1875,94 @@
       <c r="E27" s="3"/>
       <c r="F27" s="3"/>
     </row>
-    <row r="28" spans="1:6" ht="17.25" thickBot="1">
-      <c r="A28" s="18" t="s">
+    <row r="28" spans="1:6">
+      <c r="A28" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B28" s="3"/>
+      <c r="C28" s="3"/>
+      <c r="D28" s="3"/>
+      <c r="E28" s="3"/>
+      <c r="F28" s="3"/>
+    </row>
+    <row r="29" spans="1:6" ht="17.25" thickBot="1">
+      <c r="A29" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="B29" s="19" t="s">
+        <v>2</v>
+      </c>
+      <c r="C29" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="D29" s="19" t="s">
+        <v>45</v>
+      </c>
+      <c r="E29" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="F29" s="20" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6">
+      <c r="A30" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="B30" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="C30" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="B28" s="7"/>
-      <c r="C28" s="7"/>
-      <c r="D28" s="7"/>
-      <c r="E28" s="7"/>
-      <c r="F28" s="7"/>
-    </row>
-    <row r="29" spans="1:6" ht="17.25" thickBot="1">
-      <c r="A29" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="B29" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="C29" s="5" t="s">
+      <c r="D30" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="E30" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="F30" s="22" t="s">
         <v>44</v>
       </c>
-      <c r="D29" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="E29" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="F29" s="6" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" ht="17.25" thickBot="1">
-      <c r="A30" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="E30" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="F30" s="2" t="s">
-        <v>48</v>
-      </c>
     </row>
     <row r="31" spans="1:6">
-      <c r="A31" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="B31" s="15"/>
-      <c r="C31" s="15"/>
-      <c r="D31" s="15"/>
-      <c r="E31" s="15"/>
-      <c r="F31" s="15"/>
+      <c r="A31" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B31" s="3"/>
+      <c r="C31" s="3"/>
+      <c r="D31" s="3"/>
+      <c r="E31" s="3"/>
+      <c r="F31" s="3"/>
     </row>
     <row r="32" spans="1:6">
-      <c r="A32" s="13"/>
-      <c r="B32" s="13"/>
-      <c r="C32" s="13"/>
-      <c r="D32" s="13"/>
-      <c r="E32" s="13"/>
-      <c r="F32" s="13"/>
+      <c r="A32" s="3"/>
+      <c r="B32" s="3"/>
+      <c r="C32" s="3"/>
+      <c r="D32" s="3"/>
+      <c r="E32" s="3"/>
+      <c r="F32" s="3"/>
     </row>
     <row r="33" spans="1:6">
-      <c r="A33" s="13"/>
-      <c r="B33" s="13"/>
-      <c r="C33" s="16" t="s">
-        <v>41</v>
-      </c>
-      <c r="D33" s="16"/>
-      <c r="E33" s="16"/>
-      <c r="F33" s="16"/>
+      <c r="A33" s="3"/>
+      <c r="B33" s="3"/>
+      <c r="C33" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D33" s="8"/>
+      <c r="E33" s="8"/>
+      <c r="F33" s="8"/>
     </row>
     <row r="34" spans="1:6">
-      <c r="A34" s="13"/>
-      <c r="B34" s="13"/>
-      <c r="C34" s="17"/>
-      <c r="D34" s="17"/>
-      <c r="E34" s="17"/>
-      <c r="F34" s="17"/>
+      <c r="A34" s="3"/>
+      <c r="B34" s="3"/>
+      <c r="C34" s="7"/>
+      <c r="D34" s="7"/>
+      <c r="E34" s="7"/>
+      <c r="F34" s="7"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="B1:E1"/>
+  <mergeCells count="2">
     <mergeCell ref="C34:F34"/>
     <mergeCell ref="C33:F33"/>
   </mergeCells>

</xml_diff>